<commit_message>
Update script to include User Stories from Functional Specification and regenerate Excel
</commit_message>
<xml_diff>
--- a/plano_de_projeto.xlsx
+++ b/plano_de_projeto.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -916,6 +916,422 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Como um Administrador do Sistema, eu quero Gerenciar Categorias de Serviços para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>O administrador pode criar, visualizar, atualizar e inativar (soft delete) categorias que agrupam tipos de serviços.
+Fluxo Principal:
+- Administrador acessa a funcionalidade de gerenciamento de categorias.
+- Para criar: informa nome, descrição (opcional), ícone (opcional), cor (opcional), ordem e se está ativa. Sistema salva a categoria.
+- Para visualizar: Sistema exibe lista paginada de categorias com filtros (nome, ativo).
+- Para atualizar: Administrador seleciona uma categoria, modifica os campos desejados e salva.
+- Para inativar: Administrador seleciona uma categoria e confirma a inativação. Sistema marca a categoria como inativa.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Como um Administrador do Sistema, eu quero Gerenciar Tipos de Serviços para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>O administrador pode criar, visualizar, atualizar e inativar (soft delete) os tipos de serviços oferecidos, associando-os a categorias.
+Fluxo Principal:
+- Administrador acessa a funcionalidade de gerenciamento de tipos de serviços.
+- Para criar: informa categoria, código, nome, descrição (opcional), prazo estimado, valor base, e flags (requer vistoria, análise técnica, aprovação, disponível no portal, ativo). Sistema salva o tipo de serviço.
+- Para visualizar: Sistema exibe lista paginada de tipos de serviços com filtros (código, nome, categoria, disponível no portal, ativo).
+- Para atualizar: Administrador seleciona um tipo de serviço, modifica os campos desejados e salva.
+- Para inativar: Administrador seleciona um tipo de serviço e confirma a inativação.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Como um Administrador do Sistema, eu quero Gerenciar Status de Pedidos para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>O administrador pode definir os diferentes status pelos quais um pedido pode passar durante seu ciclo de vida.
+Fluxo Principal:
+- Administrador acessa a funcionalidade de gerenciamento de status de pedidos.
+- Para criar: informa código, nome, descrição (opcional), cor (opcional), ícone (opcional), ordem e se é visível no portal. Sistema salva o status.
+- Para visualizar: Sistema exibe lista paginada de status com filtros (código, nome, visível no portal).
+- Para atualizar: Administrador seleciona um status, modifica os campos desejados e salva.
+- Para inativar/excluir: Administrador seleciona um status e confirma a operação.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Como um Administrador do Sistema, eu quero Gerenciar Configurações Gerais do Sistema para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>O administrador pode gerenciar parâmetros de configuração chave-valor do sistema.
+Fluxo Principal:
+- Administrador acessa a funcionalidade de gerenciamento de configurações.
+- Para criar: informa chave, valor, descrição (opcional), tipo, grupo e se é editável. Sistema salva a configuração.
+- Para visualizar: Sistema exibe lista paginada de configurações com filtros (chave, grupo, tipo, estado).
+- Para atualizar: Administrador seleciona uma configuração, modifica os campos desejados (se editável) e salva.
+- Para inativar: Administrador seleciona uma configuração e confirma a inativação.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Como um Utente/Cidadão, Usuário Interno, eu quero Criar Pedido de Serviço para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Um utente ou um usuário interno (em nome de um utente) pode solicitar um novo serviço.
+Fluxo Principal:
+- Usuário (utente ou interno) inicia a criação de um novo pedido.
+- Seleciona o tipo de serviço desejado.
+- Informa os dados do solicitante (se usuário interno, busca/informa o cidadão).
+- Sistema registra o pedido com um status inicial (e.g., "Submetido"), data de início, e gera um código de acompanhamento.
+- (Opcional) Usuário anexa documentos iniciais.
+- Sistema notifica o usuário da criação do pedido e fornece o código de acompanhamento.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Como um Utente/Cidadão, Usuário Interno, Administrador, eu quero Acompanhar Pedido de Serviço para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Usuários podem visualizar o estado atual e o histórico de um pedido.
+Fluxo Principal:
+- Usuário busca o pedido pelo ID ou código de acompanhamento.
+- Sistema exibe os detalhes do pedido, incluindo status atual, etapa atual, datas relevantes, documentos e histórico de tramitação.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Como um Usuário Interno, Administrador, eu quero Processar Pedido de Serviço (Workflow Interno) para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Usuários internos gerenciam o fluxo do pedido, atualizando status, etapas, atribuindo responsáveis e adicionando informações. *   **Fluxo Principal (varia conforme o tipo de serviço):** 1.  Usuário interno localiza um pedido pendente. 2.  Atribui o pedido a um responsável (opcional). 3.  Analisa o pedido e os documentos. 4.  Atualiza o status e/ou etapa do pedido (e.g., "Em Análise", "Aguardando Pagamento", "Concluído"). Sistema registra no histórico. 5.  Adiciona documentos relevantes (e.g., pareceres técnicos, comprovantes). 6.  Registra informações de pagamento, se aplicável. 7.  Comunica-se com o utente se necessário (fora do escopo direto da API, mas pode ser um requisito).</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Como um Utente/Cidadão (limitado aos seus pedidos), Usuário Interno, Administrador, eu quero Gerenciar Documentos de um Pedido para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Anexar e visualizar documentos relacionados a um pedido.
+Fluxo Principal:
+- Usuário acessa um pedido específico.
+- Para anexar: seleciona o arquivo, informa nome e tipo de documento. Sistema armazena o documento (possivelmente via IGRP File Manager/MinIO) e associa ao pedido.
+- Para visualizar: Sistema lista os documentos do pedido, permitindo o download ou visualização.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Como um Utente/Cidadão (registrar pagamento para seus pedidos), Usuário Interno (confirmar/registrar pagamentos), eu quero Gerenciar Pagamentos de um Pedido para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Registrar e acompanhar o status dos pagamentos de um pedido.
+Fluxo Principal:
+- Usuário acessa um pedido que requer pagamento.
+- Para registrar: informa data do pagamento, método, referência, valor e observações. Sistema salva o pagamento.
+- Para atualizar status (interno): Usuário interno localiza o pagamento e atualiza seu status (e.g., "Confirmado", "Recusado").</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Como um Utente/Cidadão, eu quero Avaliar Pedido Concluído para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>O utente pode fornecer feedback sobre um pedido que foi concluído.
+Fluxo Principal:
+- Utente acessa um pedido concluído.
+- Sistema permite que o utente informe uma nota (e.g., de 1 a 5) e um comentário.
+- Sistema salva a avaliação. Só pode haver uma avaliação por pedido.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Como um Usuário Interno, Administrador, eu quero Gerenciar Utentes (Cidadãos/Empresas) para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Criar, visualizar, atualizar e inativar registros de utentes.
+Fluxo Principal:
+- Usuário acessa a funcionalidade de gerenciamento de utentes.
+- Para criar: informa todos os dados cadastrais relevantes (tipo de utente, identificação, nome, NIF, contatos, endereço, etc.). Sistema salva o utente.
+- Para visualizar: Sistema exibe lista paginada de utentes com filtros.
+- Para atualizar: Usuário seleciona um utente, modifica os campos desejados e salva.
+- Para inativar: Usuário seleciona um utente e confirma a inativação.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Como um Usuário Interno, Administrador, eu quero Gerenciar Serviços/Objetos Associados ao Utente para que [Benefício a ser definido/refinado].</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Associar e gerenciar serviços específicos ou objetos (como contratos, licenças) a um utente.
+Fluxo Principal:
+- Usuário acessa o cadastro de um utente.
+- Para associar serviço: informa tipo de objeto, ID do objeto (se aplicável), descrição, referência, datas, valor e estado. Sistema salva a associação.
+- Para visualizar: Sistema lista os serviços/objetos associados ao utente.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Equipa de Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>A Fazer</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>